<commit_message>
Publish Nexo UX revision c46a83b: clearer demo, PDF reports and responsive video
</commit_message>
<xml_diff>
--- a/estudio-6e94b8f2c731/archivos/Nexo-Grilla-Calendario-y-Copies.xlsx
+++ b/estudio-6e94b8f2c731/archivos/Nexo-Grilla-Calendario-y-Copies.xlsx
@@ -594,7 +594,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Pieza de Nexo: Así empieza un sistema hecho para tu empresa. Pensar que implementar un sistema exige cambiarlo todo de golpe. Ejemplo ilustrativo con datos ficticios.</t>
+          <t>Pieza de Nexo: Así empieza un sistema hecho para tu empresa. Pensar que implementar un sistema exige cambiarlo todo de golpe. Ejemplo ilustrativo con datos de demostración.</t>
         </is>
       </c>
     </row>
@@ -643,14 +643,14 @@
         <is>
           <t>Para responder por un equipo, ¿tienes que revisar varios archivos y preguntarle a alguien?
 En este ejemplo ves cómo clientes, equipos, documentos e historial se conectan en un mismo sistema. La implementación se diseña a partir de cómo funciona tu empresa y puede comenzar por un proceso.
-El video es una explicación visual con datos ficticios. Si reconoces este problema en tu operación, escríbenos por WhatsApp con la palabra CONEXIÓN y cuéntanos cómo lo gestionan hoy.</t>
+El video es una explicación visual con datos de demostración. Si reconoces este problema en tu operación, escríbenos por WhatsApp con la palabra CONEXIÓN y cuéntanos cómo lo gestionan hoy.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Un mismo equipo. Su información, en varios lugares.
 Mira cómo se conectan cliente, documentos e historial en este ejemplo de Nexo.
-Si así funciona tu empresa, escribe CONEXIÓN en el WhatsApp del perfil. Los datos del video son ficticios.
+Si así funciona tu empresa, escribe CONEXIÓN en el WhatsApp del perfil. Los datos del video son de demostración.
 #ProcesosEmpresariales #PymesPeru #GestionDeEquipos</t>
         </is>
       </c>
@@ -666,7 +666,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Pieza de Nexo: De tres escritorios a una historia conectada. Reconstruir un caso abriendo varios archivos. Ejemplo ilustrativo con datos ficticios.</t>
+          <t>Pieza de Nexo: De tres escritorios a una historia conectada. Reconstruir un caso abriendo varios archivos. Ejemplo ilustrativo con datos de demostración.</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Pieza de Nexo: Tu información existe. ¿Puedes conectarla?. Información repartida entre archivos y personas. Ejemplo ilustrativo con datos ficticios.</t>
+          <t>Pieza de Nexo: Tu información existe. ¿Puedes conectarla?. Información repartida entre archivos y personas. Ejemplo ilustrativo con datos de demostración.</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
         <is>
           <t>Encontrar un PDF resuelve una parte de la consulta. Saber a qué cliente, equipo u operación corresponde completa la respuesta.
 En Nexo trabajamos esas relaciones: que un contrato aparezca junto al alquiler al que pertenece y que el equipo conserve el vínculo con su historial.
-Este diagrama usa información ficticia para mostrar la idea. ¿Qué tipo de documento cuesta ubicar en tu empresa?</t>
+Este diagrama usa información de demostración para mostrar la idea. ¿Qué tipo de documento cuesta ubicar en tu empresa?</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Pieza de Nexo: El archivo también necesita contexto. Encontrar un PDF sin saber a qué equipo, contrato o cliente corresponde. Ejemplo ilustrativo con datos ficticios.</t>
+          <t>Pieza de Nexo: El archivo también necesita contexto. Encontrar un PDF sin saber a qué equipo, contrato o cliente corresponde. Ejemplo ilustrativo con datos de demostración.</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Pieza de Nexo: Puedes comenzar por un proceso concreto. Temor a un proyecto de software amplio e indefinido. Ejemplo ilustrativo con datos ficticios.</t>
+          <t>Pieza de Nexo: Puedes comenzar por un proceso concreto. Temor a un proyecto de software amplio e indefinido. Ejemplo ilustrativo con datos de demostración.</t>
         </is>
       </c>
     </row>
@@ -933,14 +933,14 @@
         <is>
           <t>Un equipo puede pasar por varios clientes, una devolución y un mantenimiento. Consultar solo su ubicación actual deja parte de la historia fuera.
 En este ejemplo recorremos los movimientos del mismo equipo y vemos cómo conserva el vínculo con clientes y documentos.
-Es un ejemplo de alquiler de equipos con datos ficticios. La misma lógica puede evaluarse para otros activos y procesos según el funcionamiento de cada negocio.
+Es un ejemplo de alquiler de equipos con datos de demostración. La misma lógica puede evaluarse para otros activos y procesos según el funcionamiento de cada negocio.
 Explora la demo y piensa qué historial te gustaría consultar así.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Un equipo cambia de cliente. Su historial lo acompaña.
-Devolución, mantenimiento y nuevo alquiler: mira las tres fechas de EQ-024 en este ejemplo con datos ficticios.
+Devolución, mantenimiento y nuevo alquiler: mira las tres fechas de EQ-024 en este ejemplo con datos de demostración.
 Encuentra la demo en el perfil.
 #Trazabilidad #GestionDeActivos #AlquilerDeEquipos</t>
         </is>
@@ -957,7 +957,7 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Pieza de Nexo: El equipo cambia de cliente. El historial lo acompaña.. Historial perdido o separado cada vez que se mueve un activo. Ejemplo ilustrativo con datos ficticios.</t>
+          <t>Pieza de Nexo: El equipo cambia de cliente. El historial lo acompaña.. Historial perdido o separado cada vez que se mueve un activo. Ejemplo ilustrativo con datos de demostración.</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Pieza de Nexo: ¿Cuántos archivos abres para responder por un cliente?. Información del mismo cliente fragmentada entre áreas. Ejemplo ilustrativo con datos ficticios.</t>
+          <t>Pieza de Nexo: ¿Cuántos archivos abres para responder por un cliente?. Información del mismo cliente fragmentada entre áreas. Ejemplo ilustrativo con datos de demostración.</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Pieza de Nexo: Cuando la respuesta depende de una persona. Consultas operativas que dependen de la memoria o archivos personales. Ejemplo ilustrativo con datos ficticios.</t>
+          <t>Pieza de Nexo: Cuando la respuesta depende de una persona. Consultas operativas que dependen de la memoria o archivos personales. Ejemplo ilustrativo con datos de demostración.</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1153,7 @@
           <t>¿Quién tiene este equipo? ¿Dónde estuvo antes? ¿Qué contrato le corresponde?
 En este ejemplo respondemos las tres preguntas recorriendo registros relacionados. El valor está en conservar el contexto entre clientes, equipos, movimientos y documentos.
 Diseñamos el sistema según el proceso de cada empresa. Si estas consultas hoy requieren buscar en varios lugares, escribe HISTORIA por WhatsApp y cuéntanos qué necesitas conectar.
-Demostración con datos ficticios.</t>
+Demostración con datos de demostración.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Pieza de Nexo: Tres preguntas que una ficha conectada puede responder. No poder reconstruir relaciones desde registros aislados. Ejemplo ilustrativo con datos ficticios.</t>
+          <t>Pieza de Nexo: Tres preguntas que una ficha conectada puede responder. No poder reconstruir relaciones desde registros aislados. Ejemplo ilustrativo con datos de demostración.</t>
         </is>
       </c>
     </row>
@@ -1250,7 +1250,7 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Pieza de Nexo: Tus Excels son el punto de partida. Pensar que hay que empezar desde cero o que cualquier archivo se importa sin revisión. Ejemplo ilustrativo con datos ficticios.</t>
+          <t>Pieza de Nexo: Tus Excels son el punto de partida. Pensar que hay que empezar desde cero o que cualquier archivo se importa sin revisión. Ejemplo ilustrativo con datos de demostración.</t>
         </is>
       </c>
     </row>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Pieza de Nexo: Primero el núcleo. Después, las ampliaciones.. Confundir la propuesta con campañas de WhatsApp o automatizaciones sueltas. Ejemplo ilustrativo con datos ficticios.</t>
+          <t>Pieza de Nexo: Primero el núcleo. Después, las ampliaciones.. Confundir la propuesta con campañas de WhatsApp o automatizaciones sueltas. Ejemplo ilustrativo con datos de demostración.</t>
         </is>
       </c>
     </row>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Pieza de Nexo: Muéstranos el proceso que quieres ordenar. No saber cómo iniciar una conversación sobre un sistema a medida. Ejemplo ilustrativo con datos ficticios.</t>
+          <t>Pieza de Nexo: Muéstranos el proceso que quieres ordenar. No saber cómo iniciar una conversación sobre un sistema a medida. Ejemplo ilustrativo con datos de demostración.</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Enlace a la demo; marcar “Datos ficticios”.</t>
+          <t>Enlace a la demo; marcar “Datos de demostración”.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">

</xml_diff>